<commit_message>
testing of Andreas' previous NA treatment function
</commit_message>
<xml_diff>
--- a/docs/overview_todo.xlsx
+++ b/docs/overview_todo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikto\Documents\Semester 6\Projekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikto\Documents\Semester 6\Projekt\bimi-projekt\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D464118C-9F1D-4FB3-ABCD-6A4F14190140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90057A9C-A268-4457-84DA-9B0BBD744E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{F11B7059-915B-4B83-8BD7-53D94A0E5C07}"/>
   </bookViews>
@@ -20,22 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="150">
   <si>
     <t>Bereich</t>
   </si>
@@ -375,9 +365,6 @@
     <t>Fehlerbehandlung des Datensatzes: Mindestgröße, NA-Werte, numerisch, negative Werte</t>
   </si>
   <si>
-    <t>NA-Behandlung unvollständig</t>
-  </si>
-  <si>
     <t>Funktion zur Angabe welche Gene aus einem Pathway nicht im Datensatz vorkommen</t>
   </si>
   <si>
@@ -487,6 +474,10 @@
   </si>
   <si>
     <t>Testen der Heatmap-Funktionen (kleiner Datensatz)</t>
+  </si>
+  <si>
+    <t>Rosina/
+Wiktoria</t>
   </si>
 </sst>
 </file>
@@ -556,17 +547,7 @@
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="13">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -589,16 +570,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -606,82 +577,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -776,7 +671,83 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -811,17 +782,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9DD4F59B-2EA8-4096-BCA8-9F1ED0E84D7E}" name="Tabelle1" displayName="Tabelle1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="14" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9DD4F59B-2EA8-4096-BCA8-9F1ED0E84D7E}" name="Tabelle1" displayName="Tabelle1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:H1048576" xr:uid="{9DD4F59B-2EA8-4096-BCA8-9F1ED0E84D7E}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5D447F1B-87D9-4CDF-B230-29689C0BAA81}" name="Typ" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{F9559928-FB96-4598-B354-3A6AE3B44F5B}" name="Bereich" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{DFD7A70F-970A-4A3F-8E1C-1F05FF8BA3CE}" name="Unterbereich" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{D2A919E1-344E-4D7E-BE10-6D118E8A241E}" name="Aufgabe" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{D8D64EE8-5E8B-4157-8DF2-C25CBB92469B}" name="Verantwortlich" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{C7987273-04BF-43AE-A39A-170ABC90FDC5}" name="Priorität" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{679B443A-2D07-474C-ACB4-060F822F9060}" name="Status" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{E6EF4FC0-9125-41C6-9AF0-A637BB46715F}" name="Kommentar" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{5D447F1B-87D9-4CDF-B230-29689C0BAA81}" name="Typ" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{F9559928-FB96-4598-B354-3A6AE3B44F5B}" name="Bereich" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{DFD7A70F-970A-4A3F-8E1C-1F05FF8BA3CE}" name="Unterbereich" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{D2A919E1-344E-4D7E-BE10-6D118E8A241E}" name="Aufgabe" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{D8D64EE8-5E8B-4157-8DF2-C25CBB92469B}" name="Verantwortlich" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{C7987273-04BF-43AE-A39A-170ABC90FDC5}" name="Priorität" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{679B443A-2D07-474C-ACB4-060F822F9060}" name="Status" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{E6EF4FC0-9125-41C6-9AF0-A637BB46715F}" name="Kommentar" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1193,7 +1164,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
@@ -2257,7 +2228,7 @@
         <v>12</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -2647,17 +2618,14 @@
       <c r="D65" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="E65" s="2" t="s">
-        <v>20</v>
+      <c r="E65" s="4" t="s">
+        <v>149</v>
       </c>
       <c r="F65" s="2">
         <v>1</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H65" s="4" t="s">
-        <v>112</v>
+        <v>11</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -2671,7 +2639,7 @@
         <v>82</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>30</v>
@@ -2685,16 +2653,16 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>17</v>
@@ -2717,7 +2685,7 @@
         <v>8</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>10</v>
@@ -2740,7 +2708,7 @@
         <v>8</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>10</v>
@@ -2763,7 +2731,7 @@
         <v>8</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>10</v>
@@ -2786,7 +2754,7 @@
         <v>8</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>10</v>
@@ -2809,7 +2777,7 @@
         <v>42</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>13</v>
@@ -2832,7 +2800,7 @@
         <v>42</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>13</v>
@@ -2855,7 +2823,7 @@
         <v>21</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>17</v>
@@ -2878,7 +2846,7 @@
         <v>8</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>10</v>
@@ -2890,7 +2858,7 @@
         <v>12</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -2904,7 +2872,7 @@
         <v>21</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>17</v>
@@ -2927,7 +2895,7 @@
         <v>80</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>30</v>
@@ -2941,16 +2909,16 @@
     </row>
     <row r="78" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B78" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C78" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="D78" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>129</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>54</v>
@@ -2964,16 +2932,16 @@
     </row>
     <row r="79" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C79" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D79" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>131</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>12</v>
@@ -2987,19 +2955,19 @@
     </row>
     <row r="80" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C80" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D80" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="E80" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="F80" s="2">
         <v>1</v>
@@ -3019,7 +2987,7 @@
         <v>8</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>10</v>
@@ -3042,7 +3010,7 @@
         <v>8</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>10</v>
@@ -3065,7 +3033,7 @@
         <v>8</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>10</v>
@@ -3088,7 +3056,7 @@
         <v>8</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>10</v>
@@ -3111,7 +3079,7 @@
         <v>8</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>10</v>
@@ -3134,7 +3102,7 @@
         <v>72</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>17</v>
@@ -3154,10 +3122,10 @@
         <v>36</v>
       </c>
       <c r="C87" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D87" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>17</v>
@@ -3177,10 +3145,10 @@
         <v>31</v>
       </c>
       <c r="C88" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D88" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="D88" s="5" t="s">
-        <v>147</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>30</v>
@@ -3203,7 +3171,7 @@
         <v>55</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>57</v>
@@ -3226,7 +3194,7 @@
         <v>58</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>59</v>
@@ -3239,17 +3207,17 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E1048576">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Offen">
+      <formula>NOT(ISERROR(SEARCH("Offen",E2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Fertig"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"Offen"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E1048576">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Offen">
-      <formula>NOT(ISERROR(SEARCH("Offen",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Domi's Funktion aufgerufen + Zoom funktion probiert
</commit_message>
<xml_diff>
--- a/docs/overview_todo.xlsx
+++ b/docs/overview_todo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikto\Documents\Semester 6\Projekt\bimi-projekt\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrikanarasimhan/Library/CloudStorage/OneDrive-Personal/Documents/Adri Working folder/Adrika- In progress/THI/Sem 6/Projekt/BiMi- Projekt/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ABBAB9C-FA40-4F25-9471-F0CF2177F304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2D0D87-F650-7B48-93D1-944DE2F18C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F11B7059-915B-4B83-8BD7-53D94A0E5C07}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20060" xr2:uid="{F11B7059-915B-4B83-8BD7-53D94A0E5C07}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -567,8 +567,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Gut" xfId="1" builtinId="26"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
     <dxf>
@@ -822,9 +822,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -862,7 +862,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -968,7 +968,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1110,7 +1110,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1119,20 +1119,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE99CFD6-475D-4689-869F-8F924BA3C5B8}">
   <dimension ref="A1:N90"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.46484375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.46484375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="2" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="37.1328125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="18.796875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.1640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="15" style="2" customWidth="1"/>
     <col min="8" max="8" width="48.6640625" style="4" customWidth="1"/>
-    <col min="9" max="16384" width="10.796875" style="2"/>
+    <col min="9" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -1164,7 +1164,7 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>26</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -1374,7 +1374,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>35</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
@@ -1512,7 +1512,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>26</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>26</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
@@ -1581,7 +1581,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>26</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>51</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>51</v>
       </c>
@@ -1722,7 +1722,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>51</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>26</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>33</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>51</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>26</v>
       </c>
@@ -1929,7 +1929,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>26</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>26</v>
       </c>
@@ -1998,7 +1998,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>26</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>26</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>26</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>35</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>26</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>26</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>26</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>26</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>26</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>33</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>26</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>26</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>26</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>26</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>26</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>26</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>26</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>26</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>33</v>
       </c>
@@ -2513,7 +2513,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>33</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>33</v>
       </c>
@@ -2559,7 +2559,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>26</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>26</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>33</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>26</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>26</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>113</v>
       </c>
@@ -2697,7 +2697,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>26</v>
       </c>
@@ -2720,7 +2720,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>26</v>
       </c>
@@ -2743,7 +2743,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>26</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>26</v>
       </c>
@@ -2789,7 +2789,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>26</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>26</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>26</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>26</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>33</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>26</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>113</v>
       </c>
@@ -2956,7 +2956,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>113</v>
       </c>
@@ -2979,7 +2979,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>113</v>
       </c>
@@ -3002,7 +3002,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>26</v>
       </c>
@@ -3028,7 +3028,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>26</v>
       </c>
@@ -3051,7 +3051,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>33</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>33</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>33</v>
       </c>
@@ -3117,10 +3117,10 @@
         <v>1</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.45">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>35</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>35</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>33</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>33</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
All main things completed
</commit_message>
<xml_diff>
--- a/docs/overview_todo.xlsx
+++ b/docs/overview_todo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikto\Documents\Semester 6\Projekt\bimi-projekt\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrikanarasimhan/Library/CloudStorage/OneDrive-Personal/Documents/Adri Working folder/Adrika- In progress/THI/Sem 6/Projekt/BiMi- Projekt/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4DFE74-0E36-4AF8-A7DD-CB19C090B4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23CCB58-B196-9646-B499-4F734D8F67E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F11B7059-915B-4B83-8BD7-53D94A0E5C07}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{F11B7059-915B-4B83-8BD7-53D94A0E5C07}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -612,8 +612,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Gut" xfId="1" builtinId="26"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
     <dxf>
@@ -867,9 +867,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -907,7 +907,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1013,7 +1013,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1155,7 +1155,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1164,20 +1164,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE99CFD6-475D-4689-869F-8F924BA3C5B8}">
   <dimension ref="A1:N99"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.46484375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.46484375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5" style="2" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="37.1328125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="18.796875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.1640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="15" style="2" customWidth="1"/>
     <col min="8" max="8" width="48.6640625" style="4" customWidth="1"/>
-    <col min="9" max="16384" width="10.796875" style="2"/>
+    <col min="9" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -1209,7 +1209,7 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>26</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1396,7 +1396,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>35</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
@@ -1511,7 +1511,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>26</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>26</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>26</v>
       </c>
@@ -1681,7 +1681,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>51</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>51</v>
       </c>
@@ -1773,7 +1773,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>51</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>26</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>33</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -1934,7 +1934,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>51</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>26</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>26</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>26</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>26</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>26</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>26</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>35</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>26</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>26</v>
       </c>
@@ -2230,10 +2230,10 @@
         <v>2</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.45">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2256,7 +2256,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>26</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>26</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>26</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>33</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>26</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>26</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>26</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>26</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>26</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>26</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>26</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>26</v>
       </c>
@@ -2538,7 +2538,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>33</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>33</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>33</v>
       </c>
@@ -2610,7 +2610,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>26</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>26</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>33</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>26</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>26</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>113</v>
       </c>
@@ -2748,7 +2748,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>26</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>26</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>26</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>26</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>26</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>26</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>26</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>26</v>
       </c>
@@ -2932,13 +2932,13 @@
         <v>3</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H75" s="4" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>33</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>26</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>113</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>113</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>113</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:8" ht="96" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>26</v>
       </c>
@@ -3073,13 +3073,13 @@
         <v>2</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H81" s="4" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>26</v>
       </c>
@@ -3099,10 +3099,10 @@
         <v>2</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.45">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>33</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>33</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>33</v>
       </c>
@@ -3171,7 +3171,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>35</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>35</v>
       </c>
@@ -3217,7 +3217,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>33</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>33</v>
       </c>
@@ -3263,7 +3263,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>33</v>
       </c>
@@ -3286,7 +3286,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>26</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>26</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="60.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:8" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>26</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>26</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>35</v>
       </c>
@@ -3404,7 +3404,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="61.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:8" ht="61.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>26</v>
       </c>
@@ -3424,10 +3424,10 @@
         <v>1</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.45">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>26</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>26</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
All last minute changes made (Hopefully)
</commit_message>
<xml_diff>
--- a/docs/overview_todo.xlsx
+++ b/docs/overview_todo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrikanarasimhan/Library/CloudStorage/OneDrive-Personal/Documents/Adri Working folder/Adrika- In progress/THI/Sem 6/Projekt/BiMi- Projekt/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23CCB58-B196-9646-B499-4F734D8F67E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F2665B-B636-AD4F-960C-3E01ECB42FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{F11B7059-915B-4B83-8BD7-53D94A0E5C07}"/>
   </bookViews>
@@ -851,7 +851,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9DD4F59B-2EA8-4096-BCA8-9F1ED0E84D7E}" name="Tabelle1" displayName="Tabelle1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:H1048576" xr:uid="{9DD4F59B-2EA8-4096-BCA8-9F1ED0E84D7E}"/>
+  <autoFilter ref="A1:H1048576" xr:uid="{9DD4F59B-2EA8-4096-BCA8-9F1ED0E84D7E}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Adrika"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5D447F1B-87D9-4CDF-B230-29689C0BAA81}" name="Typ" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{F9559928-FB96-4598-B354-3A6AE3B44F5B}" name="Bereich" dataDxfId="9"/>
@@ -1164,7 +1170,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE99CFD6-475D-4689-869F-8F924BA3C5B8}">
   <dimension ref="A1:N99"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.5" style="2" customWidth="1"/>
@@ -1235,7 +1241,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
@@ -1258,7 +1264,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -1281,7 +1287,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -1304,7 +1310,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
@@ -1327,7 +1333,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
@@ -1350,7 +1356,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1373,7 +1379,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -1419,7 +1425,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -1442,7 +1448,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
@@ -1465,7 +1471,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>35</v>
       </c>
@@ -1580,7 +1586,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>26</v>
       </c>
@@ -1603,7 +1609,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
@@ -1629,7 +1635,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
@@ -1704,7 +1710,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
@@ -1727,7 +1733,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>51</v>
       </c>
@@ -1750,7 +1756,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>51</v>
       </c>
@@ -1773,7 +1779,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
@@ -1796,7 +1802,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -1819,7 +1825,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>51</v>
       </c>
@@ -1842,7 +1848,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>26</v>
       </c>
@@ -1865,7 +1871,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>33</v>
       </c>
@@ -1888,7 +1894,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -1911,7 +1917,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
@@ -1934,7 +1940,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>51</v>
       </c>
@@ -1980,7 +1986,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>26</v>
       </c>
@@ -2003,7 +2009,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
@@ -2026,7 +2032,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>26</v>
       </c>
@@ -2049,7 +2055,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>26</v>
       </c>
@@ -2072,7 +2078,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>33</v>
       </c>
@@ -2095,7 +2101,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
@@ -2118,7 +2124,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>26</v>
       </c>
@@ -2141,7 +2147,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>26</v>
       </c>
@@ -2164,7 +2170,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>35</v>
       </c>
@@ -2210,7 +2216,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>26</v>
       </c>
@@ -2224,7 +2230,7 @@
         <v>86</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>10</v>
+        <v>59</v>
       </c>
       <c r="F45" s="2">
         <v>2</v>
@@ -2233,7 +2239,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2377,7 +2383,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>26</v>
       </c>
@@ -2400,7 +2406,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>26</v>
       </c>
@@ -2423,7 +2429,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>26</v>
       </c>
@@ -2446,7 +2452,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>26</v>
       </c>
@@ -2469,7 +2475,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>26</v>
       </c>
@@ -2492,7 +2498,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>26</v>
       </c>
@@ -2515,7 +2521,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>26</v>
       </c>
@@ -2538,7 +2544,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>33</v>
       </c>
@@ -2564,7 +2570,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>33</v>
       </c>
@@ -2587,7 +2593,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>33</v>
       </c>
@@ -2610,7 +2616,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>26</v>
       </c>
@@ -2633,7 +2639,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>26</v>
       </c>
@@ -2656,7 +2662,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>33</v>
       </c>
@@ -2679,7 +2685,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>26</v>
       </c>
@@ -2702,7 +2708,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>26</v>
       </c>
@@ -2725,7 +2731,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>113</v>
       </c>
@@ -2840,7 +2846,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>26</v>
       </c>
@@ -2863,7 +2869,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>26</v>
       </c>
@@ -2889,7 +2895,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>26</v>
       </c>
@@ -2938,7 +2944,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>33</v>
       </c>
@@ -2961,7 +2967,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>26</v>
       </c>
@@ -2984,7 +2990,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>113</v>
       </c>
@@ -3007,7 +3013,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>113</v>
       </c>
@@ -3030,7 +3036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>113</v>
       </c>
@@ -3171,7 +3177,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>35</v>
       </c>
@@ -3194,7 +3200,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>35</v>
       </c>
@@ -3217,7 +3223,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>33</v>
       </c>
@@ -3240,7 +3246,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>33</v>
       </c>
@@ -3263,7 +3269,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>33</v>
       </c>
@@ -3286,7 +3292,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>26</v>
       </c>
@@ -3355,7 +3361,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>26</v>
       </c>
@@ -3378,7 +3384,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>35</v>
       </c>
@@ -3427,7 +3433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>26</v>
       </c>
@@ -3453,7 +3459,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>26</v>
       </c>
@@ -3476,7 +3482,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>26</v>
       </c>

</xml_diff>